<commit_message>
fix(attestation): include store managers in wave notifications, populate manager questions and fix duration to 1 day
</commit_message>
<xml_diff>
--- a/template_attestation.xlsx
+++ b/template_attestation.xlsx
@@ -621,7 +621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -683,41 +683,459 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Зразкове питання для посади Керівник?</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Варіант А</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Варіант Б (Правильний)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Варіант В</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Варіант Г</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Пояснення чому відповідь 2 вірна.</t>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Яка першочергова дія керівника пекарні при відкритті зміни перед допуском персоналу до роботи?</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Почати випікати здобу</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Перевірити наявність та чинність медичних книжок, стан здоров'я працівників та відповідність фірмовому одягу</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Замовити рекламу в соціальних мережах</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Перерахувати весь залишок борошна на складі</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>За вимогами НАССР та корпоративними стандартами керівник зобов'язаний провести візуальний огляд персоналу (відсутність симптомів ГРВІ/порізів), перевірити санітарний одяг та допуск до роботи.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Який допустимий температурний режим у холодильних вітринах для кондитерських виробів та кулінарії?</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>-5...+0°C</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>+2...+6°C</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>+8...+12°C</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>+15...+18°C</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Стандартний температурний режим зберігання та експозиції кондитерських виробів та готової кулінарії становить +2...+6°C. Дані фіксуються в журналі температурного контролю.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>У разі раптового зникнення електроенергії в пекарні, які дії керівника є правильними щодо продукції в холодильниках?</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Негайно відкрити всі холодильники для провітрювання</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Тримати холодильні та морозильні камери щільно закритими для збереження холоду, зафіксувати час відключення</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Списати всю продукцію через 15 хвилин</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Перенести продукцію на звичайні столи в торговий зал</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Закриті холодильники здатні утримувати безпечну температуру протягом кількох годин. Керівник фіксує час відключення, повідомляє техпідтримку і мінімізує відкриття дверей камер.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Як оформлюється списання бракованої або продукції з вичерпаним терміном придатності?</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Продукція просто викидається у смітник без записів</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Складається Акт списання із зазначенням причини, найменування, ваги/кількості та підписом комісії</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Продукція роздається безкоштовно персоналу</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Продукція переробляється у новий виріб без маркування</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Будь-яке списання продукції здійснюється виключно за встановленим внутрішнім регламентом через офіційний Акт списання в обліковій програмі.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Який порядок дій керівника при виявленні невідповідності (браку) у партії заморожених напівфабрикатів від постачальника?</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Прийняти товар і спробувати використати самостійно</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Скласти Акт розбіжностей/претензію, сфотографувати брак, повернути або ізолювати партію з маркуванням 'Брак'</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Оштрафувати водія на місці готівкою</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Знищити партію товару без повідомлення постачальника</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Прийом неякісної сировини заборонено. Складається офіційний акт із фотофіксацією, товар ізолюється з маркуванням або повертається постачальнику.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Що повинен зробити керівник при виявленні нестачі або надлишку готівки в касі під час вечірньої інкасації?</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Покрити нестачу з власної кишені або забрати надлишок собі</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Провести перерахунок, зняти X-звіт, з'ясувати причину розбіжності з касиром та скласти пояснювальну записку</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Не знімати Z-звіт і залишити касу відкритою</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Звільнити касира без з'ясування причин</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Касова дисципліна вимагає документального підтвердження: повторний перерахунок купюр, аналіз чеків повернення/корекції, оформлення пояснювальної та відповідного акту розбіжностей.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Який максимальний термін перебування стажера на випробувальному терміні до прийняття рішення про атестацію/переведення?</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>1 день</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>5 днів (згідно з навчальною програмою платформи BULKA)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>6 місяців</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Термін необмежений</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Базовий навчальний курс та стажування в BULKA розраховані на 5 навчальних днів, після чого керівник оцінює практичні навички та приймає рішення про переведення в статус 'Працівник'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Як діяти керівнику, якщо гість поводиться агресивно та вимагає негайного повернення коштів за напій/страву?</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Відповісти агресією та викликати охорону без розмов</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Зберігати спокій, вислухати гостя без перебивання, запропонувати переробити напій або оформити повернення коштів</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Ігнорувати гостя і піти в службове приміщення</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Змусити працівника оплатити рахунок гостя</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Стандарт деескалації конфліктів: активне слухання, прояв турботи, доброзичливе виправлення ситуації (заміна або повернення коштів згідно з чеком).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Яка періодичність проведення генерального прибирання та дезінфекції в пекарні згідно з санітарними нормами?</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Раз на рік</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Щотижня за графіком із заповненням санітарного журналу</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Тільки перед приїздом перевірки</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Генеральне прибирання не обов'язкове при щоденному підмітанні</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Генеральне прибирання всіх поверхонь, миття холодильного обладнання, стелажів та вентиляції проводиться щотижня за затвердженим графіком із відміткою в журналі НАССР.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Які зобов'язання керівника щодо обліку робочого часу персоналу пекарні?</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Облік не потрібен, якщо працівники приходять вчасно</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Щоденне точне ведення табеля робочого часу (вихід, запізнення, відпрацьовані години, лікарняні)</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Записувати години раз на місяць приблизно по пам'яті</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Довірити заповнення табеля кожному стажеру самостійно</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Керівник несе персональну відповідальність за своєчасне та достовірне ведення табеля обліку робочого часу (ТОРВ) своєї торгової точки.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Що робити керівнику у разі виявлення протермінованого дезінфікуючого засобу для поверхонь?</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Продовжувати використовувати, збільшивши концентрацію</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Негайно вилучити з використання, утилізувати та замовити свіжу сертифіковану хімію</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Змішати з іншим миючим засобом</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Використовувати звичайну воду</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Протерміновані деззасоби втрачають бактерицидні властивості, що загрожує харчовій безпеці. Засіб вилучається і замінюється згідно зі стандартами НАССР.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Який порядок дій керівника, якщо на зміну не вийшов основний касир чи пекар?</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Закрити магазин на цілий день без попередження</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>З'ясувати причину, оперативно організувати заміну із резерву або перерозподілити обов'язки та повідомити територіала</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Змусити стажера працювати без навчання</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Не вживати жодних дій</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Керівник оперативно координує безперебійну роботу пекарні: зв'язується із підмінними співробітниками або територіальним менеджером для забезпечення робочого графіка.</t>
         </is>
       </c>
     </row>

</xml_diff>